<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.001-06 Le garage de la planche
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.001-06.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.001-06.xlsx
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Raphaël, Chouchou, papa</t>
+          <t>Raphaël, Chouchou, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Raphaël veut un garage pour le camion, avec la caisse et la planche. Le toit est trop haut pour Chouchou. Ils baissent un bord. Le camion rentre.</t>
+          <t>Un torchon orange claque au fil. Sur le bord, un éclat de planche brille. Raphaël veut un garage pour le camion, maintenant, avec la caisse et la planche. Il pose trop haut : Chouchou n'atteint pas. Le camion tape. Sourire parti. Il refuse de foncer, baisse un bord. Ils jouent. Merci vécu. Il relève trop vite : ça glisse. Il refuse, baisse avec elle. L'éclat de planche tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La planche sent la résine. Elle est chaude du soleil. Un fil à linge fait de l'ombre. Le linge claque un peu. Une caisse de bois attend. Dedans, un camion de bois dort. Tu as senti la planche, Raphaël ? Oui, papa. Elle sent l'arbre. Oui. Je veux un garage pour le camion. Avec la caisse et la planche ? Oui. En ce moment, Raphaël ouvre la caisse. Le bois est lisse, un peu chaud. Chouchou arrive sur les dalles. Chouchou est plus petit. Raphaël est plus grand. Ils ont des tailles différentes. Chouchou, tu veux le garage ? Oui. Vous jouez ensemble. On peut jouer ensemble. Raphaël pose la planche sur la caisse. Le toit est haut. Chouchou pousse le camion. Le camion n'entre pas. C'est trop haut. On baisse un côté, alors. Papa pose un livre sous un bord. L'autre bord reste sur la caisse. Le toit penche, tout doux. Il entre, maintenant ? On essaie. Une fourmi croise la terrasse. Elle contourne la caisse. On laisse la fourmi ? Oui. Le linge fait une ombre mobile. Elle passe sur le camion. Le garage a du soleil. Et de l'ombre, aussi.</t>
+          <t>Un torchon orange claque au fil. Il claque, papa ! Tu l'entends, dans le vent ? Oui, un son court. L'air du soir sent la résine, un peu tiède. Ça sent l'arbre, maman. Tu le sens, près de la planche ? Oui, maman. La planche de résine attend contre la caisse. Sur le bord, un éclat de planche brille. Il brille, papa. C'est le soir, sur la résine ? Oui, un petit point. Les dalles de la terrasse sont fraîches. Elles piquent les pieds. On reste près de la caisse ? Oui, maman. La lumière orange glisse sur les dalles. Elle est chaude, plus loin. Le vent bouge le fil, Raphaël. Oui, papa. Une caisse de bois attend près du mur. Dedans, un camion de bois dort. Le camion ! Ses roues sont rouges. Tu le sors, Raphaël ? Oui, papa. Raphaël sort le camion de la caisse. Le bois est lisse, un peu chaud. Je veux un garage, maintenant ! Avec la caisse et la planche ? Oui, maman. Le toit, c'est la planche ? Oui, papa. Maman accroche un torchon au fil. Le fil tient, ce soir. Il bouge. Chouchou arrive sur les dalles. Ses mains pendent plus bas, près du fil. Chouchou ! J'arrive. Le garage, maintenant, Chouchou ! En ce moment, Raphaël pose la planche trop haut. La planche tape le bord de la caisse. Pousse, tout de suite ! Raphaël attrape la manche de Chouchou. Non. Chouchou recule vers le fil. Oh. Chouchou pousse le camion, un peu. Le camion tape le toit trop haut. C'est trop haut ! Mes mains n'arrivent pas. Le camion reste dehors, contre le bois. Oh. L'éclat de planche tremble, puis tient. Il part. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Le toit est haut, Raphaël ? Papa s'accroupit à la même hauteur. Oui, papa. La phrase se perd dans le vent du soir. Personne n'entend la fin. Chouchou est près du fil, Raphaël. Oui, maman. Le camion reste lourd, entre leurs pieds.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La planche sent la résine. Elle est chaude du soleil. Un fil à linge fait de l'ombre. Le linge claque un peu. Une caisse de bois attend. Dedans, un camion de bois dort. Tu as senti la planche, Raphaël ? Oui, papa. Elle sent l'arbre. Oui. Je veux un garage pour le camion. Avec la caisse et la planche ? Oui. En ce moment, Raphaël ouvre la caisse. Le bois est lisse, un peu chaud. Chouchou arrive sur les dalles. Chouchou est plus petit. Raphaël est plus grand. Ils ont des tailles différentes. Chouchou, tu veux le garage ? Oui. Vous jouez ensemble. On peut jouer ensemble. Raphaël pose la planche sur la caisse. Le toit est haut. Chouchou pousse le camion. Le camion n'entre pas. C'est trop haut. On baisse un côté, alors. Papa pose un livre sous un bord. L'autre bord reste sur la caisse. Le toit penche, tout doux. Il entre, maintenant ? On essaie. Une fourmi croise la terrasse. Elle contourne la caisse. On laisse la fourmi ? Oui. Le linge fait une ombre mobile. Elle passe sur le camion. Le garage a du soleil. Et de l'ombre, aussi.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un torchon orange claque au fil. Il claque, papa ! Tu l'entends, dans le vent ? Oui, un son court. L'air du soir sent la résine, un peu tiède. Ça sent l'arbre, maman. Tu le sens, près de la planche ? Oui, maman. La planche de résine attend contre la caisse. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat de planche&lt;/emphasis&gt; brille. Il brille, papa. C'est le soir, sur la résine ? Oui, un petit point. Les dalles de la terrasse sont fraîches. Elles piquent les pieds. On reste près de la caisse ? Oui, maman. La lumière orange glisse sur les dalles. Elle est chaude, plus loin. Le vent bouge le fil, Raphaël. Oui, papa. Une caisse de bois attend près du mur. Dedans, un camion de bois dort. Le camion ! Ses roues sont rouges. Tu le sors, Raphaël ? Oui, papa. Raphaël sort le camion de la caisse. Le bois est lisse, un peu chaud. Je veux un garage, maintenant ! Avec la caisse et la planche ? Oui, maman. Le toit, c'est la planche ? Oui, papa. Maman accroche un torchon au fil. Le fil tient, ce soir. Il bouge. Chouchou arrive sur les dalles. Ses mains pendent plus bas, près du fil. Chouchou ! J'arrive. Le garage, maintenant, Chouchou ! En ce moment, Raphaël pose la planche trop haut. La planche tape le bord de la caisse. Pousse, tout de suite ! Raphaël attrape la manche de Chouchou. Non. Chouchou recule vers le fil. Oh. Chouchou pousse le camion, un peu. Le camion tape le toit trop haut. C'est trop haut ! Mes mains n'arrivent pas. Le camion reste dehors, contre le bois. Oh. L'éclat de planche tremble, puis tient. Il part. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Le toit est haut, Raphaël ? Papa s'accroupit à la même hauteur. Oui, papa. La phrase se perd dans le vent du soir. Personne n'entend la fin. Chouchou est près du fil, Raphaël. Oui, maman. Le camion reste lourd, entre leurs pieds.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Titouan et Romane sont au jardin avec papa. Romane est plus petite. Titouan est plus grand. Papa dit : les &lt;emphasis&gt;tailles&lt;/emphasis&gt; sont différentes. On joue ensemble. Titouan n'invente pas de surnom. Il tend un cube. Romane pose un cube. Ils construisent une tour. Papa dit : on joue ensemble. Plus petit ou plus grand, on joue. [pause]</t>
+          <t>Un torchon orange claque au fil. Il claque, papa ! Tu l'entends, dans le vent ? Oui, un son court. L'air du soir sent la résine, un peu tiède. Ça sent l'arbre, maman. Tu le sens, près de la planche ? Oui, maman. La planche de résine attend contre la caisse. Sur le bord, un &lt;emphasis&gt;éclat de planche&lt;/emphasis&gt; brille. Il brille, papa. C'est le soir, sur la résine ? Oui, un petit point. Les dalles de la terrasse sont fraîches. Elles piquent les pieds. On reste près de la caisse ? Oui, maman. La lumière orange glisse sur les dalles. Elle est chaude, plus loin. Le vent bouge le fil, Raphaël. Oui, papa. Une caisse de bois attend près du mur. Dedans, un camion de bois dort. Le camion ! Ses roues sont rouges. Tu le sors, Raphaël ? Oui, papa. Raphaël sort le camion de la caisse. Le bois est lisse, un peu chaud. Je veux un garage, maintenant ! Avec la caisse et la planche ? Oui, maman. Le toit, c'est la planche ? Oui, papa. Maman accroche un torchon au fil. Le fil tient, ce soir. Il bouge. Chouchou arrive sur les dalles. Ses mains pendent plus bas, près du fil. Chouchou ! J'arrive. Le garage, maintenant, Chouchou ! En ce moment, Raphaël pose la planche trop haut. La planche tape le bord de la caisse. Pousse, tout de suite ! Raphaël attrape la manche de Chouchou. Non. Chouchou recule vers le fil. Oh. Chouchou pousse le camion, un peu. Le camion tape le toit trop haut. C'est trop haut ! Mes mains n'arrivent pas. Le camion reste dehors, contre le bois. Oh. L'éclat de planche tremble, puis tient. Il part. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Le toit est haut, Raphaël ? Papa s'accroupit à la même hauteur. Oui, papa. La phrase se perd dans le vent du soir. Personne n'entend la fin. Chouchou est près du fil, Raphaël. Oui, maman. Le camion reste lourd, entre leurs pieds. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>tailles</t>
+          <t>éclat de planche</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,51 +1326,85 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_garage_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La planche sent la résine.
-narrateur|Elle est chaude du soleil.
-narrateur|Un fil à linge fait de l'ombre.
-narrateur|Le linge claque un peu.
-narrateur|Une caisse de bois attend.
+          <t>narrateur|Un torchon orange claque au fil.
+enfant-m|Il claque, papa !
+papa|Tu l'entends, dans le vent ?
+enfant-m|Oui, un son court.
+narrateur|L'air du soir sent la résine, un peu tiède.
+enfant-m|Ça sent l'arbre, maman.
+maman|Tu le sens, près de la planche ?
+enfant-m|Oui, maman.
+narrateur|La planche de résine attend contre la caisse.
+narrateur|Sur le bord, un éclat de planche brille.
+enfant-m|Il brille, papa.
+papa|C'est le soir, sur la résine ?
+enfant-m|Oui, un petit point.
+narrateur|Les dalles de la terrasse sont fraîches.
+enfant-m|Elles piquent les pieds.
+maman|On reste près de la caisse ?
+enfant-m|Oui, maman.
+narrateur|La lumière orange glisse sur les dalles.
+enfant-m|Elle est chaude, plus loin.
+papa|Le vent bouge le fil, Raphaël.
+enfant-m|Oui, papa.
+narrateur|Une caisse de bois attend près du mur.
 narrateur|Dedans, un camion de bois dort.
-papa|Tu as senti la planche, Raphaël ?
+enfant-m|Le camion !
+enfant-m|Ses roues sont rouges.
+papa|Tu le sors, Raphaël ?
 enfant-m|Oui, papa.
-enfant-m|Elle sent l'arbre.
-papa|Oui.
-enfant-m|Je veux un garage pour le camion.
-papa|Avec la caisse et la planche ?
-enfant-m|Oui.
-narrateur|En ce moment, Raphaël ouvre la caisse.
+narrateur|Raphaël sort le camion de la caisse.
 narrateur|Le bois est lisse, un peu chaud.
+enfant-m|Je veux un garage, maintenant !
+maman|Avec la caisse et la planche ?
+enfant-m|Oui, maman.
+papa|Le toit, c'est la planche ?
+enfant-m|Oui, papa.
+narrateur|Maman accroche un torchon au fil.
+maman|Le fil tient, ce soir.
+enfant-m|Il bouge.
 narrateur|Chouchou arrive sur les dalles.
-narrateur|Chouchou est plus petit.
-narrateur|Raphaël est plus grand.
-narrateur|Ils ont des tailles différentes.
-enfant-m|Chouchou, tu veux le garage ?
-copain|Oui.
-papa|Vous jouez ensemble.
-papa|On peut jouer ensemble.
-narrateur|Raphaël pose la planche sur la caisse.
-narrateur|Le toit est haut.
-narrateur|Chouchou pousse le camion.
-narrateur|Le camion n'entre pas.
-enfant-m|C'est trop haut.
-papa|On baisse un côté, alors.
-narrateur|Papa pose un livre sous un bord.
-narrateur|L'autre bord reste sur la caisse.
-narrateur|Le toit penche, tout doux.
-copain|Il entre, maintenant ?
-enfant-m|On essaie.
-narrateur|Une fourmi croise la terrasse.
-narrateur|Elle contourne la caisse.
-papa|On laisse la fourmi ?
-enfant-m|Oui.
-narrateur|Le linge fait une ombre mobile.
-narrateur|Elle passe sur le camion.
-enfant-m|Le garage a du soleil.
-papa|Et de l'ombre, aussi.</t>
+narrateur|Ses mains pendent plus bas, près du fil.
+enfant-m|Chouchou !
+enfant-f|J'arrive.
+enfant-m|Le garage, maintenant, Chouchou !
+narrateur|En ce moment, Raphaël pose la planche trop haut.
+narrateur|La planche tape le bord de la caisse.
+enfant-m|Pousse, tout de suite !
+narrateur|Raphaël attrape la manche de Chouchou.
+enfant-f|Non.
+narrateur|Chouchou recule vers le fil.
+enfant-m|Oh.
+narrateur|Chouchou pousse le camion, un peu.
+narrateur|Le camion tape le toit trop haut.
+enfant-m|C'est trop haut !
+enfant-f|Mes mains n'arrivent pas.
+narrateur|Le camion reste dehors, contre le bois.
+enfant-m|Oh.
+narrateur|L'éclat de planche tremble, puis tient.
+enfant-m|Il part.
+narrateur|Le sourire de Raphaël disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+papa|Le toit est haut, Raphaël ?
+narrateur|Papa s'accroupit à la même hauteur.
+enfant-m|Oui, papa.
+narrateur|La phrase se perd dans le vent du soir.
+narrateur|Personne n'entend la fin.
+maman|Chouchou est près du fil, Raphaël.
+enfant-m|Oui, maman.
+narrateur|Le camion reste lourd, entre leurs pieds.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>linge,planche</t>
         </is>
       </c>
     </row>
@@ -1402,12 +1436,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Chouchou est plus petit. Que fait Raphaël ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Chouchou est plus petit. Que fait &lt;emphasis level="moderate"&gt;Raphaël&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Romane est plus petite. Que fait Titouan ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Chouchou est plus petit. Que fait &lt;emphasis&gt;Raphaël&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1470,7 +1504,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1478,10 +1512,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1496,34 +1530,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Raphaël</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1532,23 +1570,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_joue_avec_elle_sans_poser_trop_haut; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1581,17 +1619,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou pousse le camion. Le camion rentre sous la planche. Les roues font un petit clic. Il est dedans ! Oui. Les deux façons marchent. Raphaël pose un cube en enseigne. Chouchou pose une feuille devant. C'est la porte, tout doux. Le camion dort. Il est au garage. Vous avez des tailles différentes. Et vous jouez ensemble. Le garage est solide, non ? Oui, papa. La fourmi contourne le cube. Chouchou la suit des yeux. Le linge claque encore une fois. La planche sent toujours la résine. Encore un voyage ? Un tout petit. Le camion sort, puis rentre. Le toit ne bouge plus. Vous construisez ensemble.</t>
+          <t>Raphaël pose la planche trop haut, une fois. Pousse, Chouchou, maintenant ! Les mots se bousculent dans sa bouche. Non. Chouchou reste près du fil. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il lâche la manche, un peu. Le toit est haut, Raphaël ? Papa reste à sa hauteur. Les mains de Chouchou n'arrivent pas. Maman n'a pas fini non plus. Raphaël attend que le silence arrive. On joue, Chouchou ? Plus bas, si tu veux ? Chouchou ne dit rien. Elle regarde le camion, longtemps. Je regarde. D'accord. Raphaël baisse un bord de la planche. L'autre bord reste sur la caisse. Le toit penche, assez bas. Je pousse. Chouchou pousse le camion sans presser. Les roues font un petit clic. Il est dedans ! Merci, Raphaël. Papa a entendu toute la phrase. Tu tiens le bord, des deux mains ? Oui, maman. Le camion est au garage. Tu as entendu les roues ? Oui, papa. On reste à la terrasse, Raphaël ? Oui. Le camion sent le bois, un peu tiède. Il colle aux doigts. Comme la résine, oui.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou pousse le camion. Le camion rentre sous la planche. Les roues font un petit clic. Il est dedans ! Oui. Les deux façons marchent. Raphaël pose un cube en enseigne. Chouchou pose une feuille devant. C'est la porte, tout doux. Le camion dort. Il est au garage. Vous avez des tailles différentes. Et vous jouez ensemble. Le garage est solide, non ? Oui, papa. La fourmi contourne le cube. Chouchou la suit des yeux. Le linge claque encore une fois. La planche sent toujours la résine. Encore un voyage ? Un tout petit. Le camion sort, puis rentre. Le toit ne bouge plus. Vous construisez ensemble.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël pose la planche trop haut, une fois. Pousse, Chouchou, maintenant ! Les mots se bousculent dans sa bouche. Non. Chouchou reste près du fil. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il lâche la manche, un peu. Le toit est haut, Raphaël ? Papa reste à sa hauteur. Les mains de Chouchou n'arrivent pas. Maman n'a pas fini non plus. Raphaël attend que le silence arrive. &lt;emphasis level="moderate"&gt;On joue&lt;/emphasis&gt;, Chouchou ? Plus bas, si tu veux ? Chouchou ne dit rien. Elle regarde le camion, longtemps. Je regarde. D'accord. Raphaël baisse un bord de la planche. L'autre bord reste sur la caisse. Le toit penche, assez bas. Je pousse. Chouchou pousse le camion sans presser. Les roues font un petit clic. Il est dedans ! Merci, Raphaël. Papa a entendu toute la phrase. Tu tiens le bord, des deux mains ? Oui, maman. Le camion est au garage. Tu as entendu les roues ? Oui, papa. On reste à la terrasse, Raphaël ? Oui. Le camion sent le bois, un peu tiède. Il colle aux doigts. Comme la résine, oui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Titouan a joué avec Romane. &lt;emphasis&gt;tailles&lt;/emphasis&gt; différentes. On joue ensemble. [pause]</t>
+          <t>Raphaël pose la planche trop haut, une fois. Pousse, Chouchou, maintenant ! Les mots se bousculent dans sa bouche. Non. Chouchou reste près du fil. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il lâche la manche, un peu. Le toit est haut, Raphaël ? Papa reste à sa hauteur. Les mains de Chouchou n'arrivent pas. Maman n'a pas fini non plus. Raphaël attend que le silence arrive. &lt;emphasis&gt;On joue&lt;/emphasis&gt;, Chouchou ? Plus bas, si tu veux ? Chouchou ne dit rien. Elle regarde le camion, longtemps. Je regarde. D'accord. Raphaël baisse un bord de la planche. L'autre bord reste sur la caisse. Le toit penche, assez bas. Je pousse. Chouchou pousse le camion sans presser. Les roues font un petit clic. Il est dedans ! Merci, Raphaël. Papa a entendu toute la phrase. Tu tiens le bord, des deux mains ? Oui, maman. Le camion est au garage. Tu as entendu les roues ? Oui, papa. On reste à la terrasse, Raphaël ? Oui. Le camion sent le bois, un peu tiède. Il colle aux doigts. Comme la résine, oui. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1638,7 +1676,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1646,10 +1684,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1672,30 +1710,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>tailles</t>
+          <t>On joue</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1704,10 +1742,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1720,35 +1758,55 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_baisse_le_toit_ils_jouent; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou pousse le camion.
-narrateur|Le camion rentre sous la planche.
+          <t>narrateur|Raphaël pose la planche trop haut, une fois.
+enfant-m|Pousse, Chouchou, maintenant !
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-f|Non.
+narrateur|Chouchou reste près du fil.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Raphaël refuse de foncer.
+narrateur|Il lâche la manche, un peu.
+papa|Le toit est haut, Raphaël ?
+narrateur|Papa reste à sa hauteur.
+maman|Les mains de Chouchou n'arrivent pas.
+narrateur|Maman n'a pas fini non plus.
+narrateur|Raphaël attend que le silence arrive.
+enfant-m|On joue, Chouchou ?
+enfant-m|Plus bas, si tu veux ?
+narrateur|Chouchou ne dit rien.
+narrateur|Elle regarde le camion, longtemps.
+enfant-f|Je regarde.
+enfant-m|D'accord.
+narrateur|Raphaël baisse un bord de la planche.
+narrateur|L'autre bord reste sur la caisse.
+narrateur|Le toit penche, assez bas.
+enfant-f|Je pousse.
+narrateur|Chouchou pousse le camion sans presser.
 narrateur|Les roues font un petit clic.
 enfant-m|Il est dedans !
-papa|Oui.
-papa|Les deux façons marchent.
-narrateur|Raphaël pose un cube en enseigne.
-narrateur|Chouchou pose une feuille devant.
-narrateur|C'est la porte, tout doux.
-copain|Le camion dort.
-enfant-m|Il est au garage.
-papa|Vous avez des tailles différentes.
-papa|Et vous jouez ensemble.
-papa|Le garage est solide, non ?
+papa|Merci, Raphaël.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu tiens le bord, des deux mains ?
+enfant-m|Oui, maman.
+enfant-f|Le camion est au garage.
+papa|Tu as entendu les roues ?
 enfant-m|Oui, papa.
-narrateur|La fourmi contourne le cube.
-narrateur|Chouchou la suit des yeux.
-narrateur|Le linge claque encore une fois.
-narrateur|La planche sent toujours la résine.
-enfant-m|Encore un voyage ?
-copain|Un tout petit.
-narrateur|Le camion sort, puis rentre.
-narrateur|Le toit ne bouge plus.
-papa|Vous construisez ensemble.</t>
+maman|On reste à la terrasse, Raphaël ?
+enfant-m|Oui.
+narrateur|Le camion sent le bois, un peu tiède.
+enfant-m|Il colle aux doigts.
+maman|Comme la résine, oui.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>roues</t>
         </is>
       </c>
     </row>
@@ -1775,17 +1833,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On range le camion dans la caisse ? Oui. Raphaël glisse le camion. Chouchou pose la feuille à côté. Papa pose la planche contre le mur. Tu as fini de ranger le camion ? Oui, papa. Le linge bouge encore, au vent. Les dalles redeviennent calmes. On se lave les mains ? Oui. Le soleil du soir baisse un peu. L'ombre du fil s'allonge.</t>
+          <t>Raphaël veut un toit plus haut. Un grand garage, maintenant ! Il relève la planche trop vite. Le toit glisse sur la caisse. Oh. Le camion tape le bord, puis recule. Il sort. Oh. Les deux voix se mélangent. La planche glisse, Raphaël. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Il écoute la terrasse, un instant. Il observe la planche, écoute le fil. Sur le bord, un éclat de planche luit. Il est là. On baisse, si tu veux ? Plus tard. D'accord. Chouchou s'approche, sans se presser. Raphaël baisse le bord, avec elle. Le toit penche, assez bas pour deux. Je pousse. Les roues passent sous la planche. Ça fait toc. Il est dedans. Tu restes un peu ? Oui, papa. La planche est près de la caisse. On la laisse ? Oui, contre le bois. Un cube jaune attend près du mur. L'enseigne, plus bas ? Oui. Ils posent le cube devant la caisse. C'est la porte, Chouchou. Le camion dort. Le fil claque, au vent. Je l'entends.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On range le camion dans la caisse ? Oui. Raphaël glisse le camion. Chouchou pose la feuille à côté. Papa pose la planche contre le mur. Tu as fini de ranger le camion ? Oui, papa. Le linge bouge encore, au vent. Les dalles redeviennent calmes. On se lave les mains ? Oui. Le soleil du soir baisse un peu. L'ombre du fil s'allonge.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël veut un toit plus haut. Un grand garage, maintenant ! Il relève la planche trop vite. Le toit glisse sur la caisse. Oh. Le camion tape le bord, puis recule. Il sort. Oh. Les deux voix se mélangent. La planche glisse, Raphaël. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Il écoute la terrasse, un instant. Il observe la planche, écoute le fil. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat de planche&lt;/emphasis&gt; luit. Il est là. On baisse, si tu veux ? Plus tard. D'accord. Chouchou s'approche, sans se presser. Raphaël baisse le bord, avec elle. Le toit penche, assez bas pour deux. Je pousse. Les roues passent sous la planche. Ça fait toc. Il est dedans. Tu restes un peu ? Oui, papa. La planche est près de la caisse. On la laisse ? Oui, contre le bois. Un cube jaune attend près du mur. L'enseigne, plus bas ? Oui. Ils posent le cube devant la caisse. C'est la porte, Chouchou. Le camion dort. Le fil claque, au vent. Je l'entends.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Papa range les cubes. Titouan donne la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Raphaël veut un toit plus haut. Un grand garage, maintenant ! Il relève la planche trop vite. Le toit glisse sur la caisse. Oh. Le camion tape le bord, puis recule. Il sort. Oh. Les deux voix se mélangent. La planche glisse, Raphaël. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Il écoute la terrasse, un instant. Il observe la planche, écoute le fil. Sur le bord, un &lt;emphasis&gt;éclat de planche&lt;/emphasis&gt; luit. Il est là. On baisse, si tu veux ? Plus tard. D'accord. Chouchou s'approche, sans se presser. Raphaël baisse le bord, avec elle. Le toit penche, assez bas pour deux. Je pousse. Les roues passent sous la planche. Ça fait toc. Il est dedans. Tu restes un peu ? Oui, papa. La planche est près de la caisse. On la laisse ? Oui, contre le bois. Un cube jaune attend près du mur. L'enseigne, plus bas ? Oui. Ils posent le cube devant la caisse. C'est la porte, Chouchou. Le camion dort. Le fil claque, au vent. Je l'entends. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1832,7 +1890,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1840,10 +1898,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1866,30 +1924,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de planche</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1898,10 +1956,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1912,22 +1970,57 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_sur_le_toit; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>papa|On range le camion dans la caisse ?
-enfant-m|Oui.
-narrateur|Raphaël glisse le camion.
-narrateur|Chouchou pose la feuille à côté.
-narrateur|Papa pose la planche contre le mur.
-papa|Tu as fini de ranger le camion ?
+          <t>narrateur|Raphaël veut un toit plus haut.
+enfant-m|Un grand garage, maintenant !
+narrateur|Il relève la planche trop vite.
+narrateur|Le toit glisse sur la caisse.
+enfant-m|Oh.
+narrateur|Le camion tape le bord, puis recule.
+enfant-f|Il sort.
+enfant-m|Oh.
+narrateur|Les deux voix se mélangent.
+papa|La planche glisse, Raphaël.
+narrateur|Raphaël refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Il écoute la terrasse, un instant.
+narrateur|Il observe la planche, écoute le fil.
+narrateur|Sur le bord, un éclat de planche luit.
+enfant-m|Il est là.
+enfant-m|On baisse, si tu veux ?
+enfant-f|Plus tard.
+enfant-m|D'accord.
+narrateur|Chouchou s'approche, sans se presser.
+narrateur|Raphaël baisse le bord, avec elle.
+narrateur|Le toit penche, assez bas pour deux.
+enfant-f|Je pousse.
+narrateur|Les roues passent sous la planche.
+narrateur|Ça fait toc.
+enfant-m|Il est dedans.
+papa|Tu restes un peu ?
 enfant-m|Oui, papa.
-narrateur|Le linge bouge encore, au vent.
-narrateur|Les dalles redeviennent calmes.
-papa|On se lave les mains ?
-enfant-m|Oui.
-narrateur|Le soleil du soir baisse un peu.
-narrateur|L'ombre du fil s'allonge.</t>
+maman|La planche est près de la caisse.
+enfant-m|On la laisse ?
+papa|Oui, contre le bois.
+narrateur|Un cube jaune attend près du mur.
+enfant-m|L'enseigne, plus bas ?
+enfant-f|Oui.
+narrateur|Ils posent le cube devant la caisse.
+enfant-m|C'est la porte, Chouchou.
+enfant-f|Le camion dort.
+maman|Le fil claque, au vent.
+enfant-m|Je l'entends.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>linge</t>
         </is>
       </c>
     </row>
@@ -1954,17 +2047,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le camion a eu un garage. On a joué ensemble. Bravo, Raphaël. La planche sent encore la résine.</t>
+          <t>Ils restent près de la caisse. Maman referme le bord, sans bruit. Comme un toit, papa. Tu le vois, toi ? Oui, sur le bord. On est bien, ici. Raphaël glisse le doigt, sans se presser. On le sent, maman. Tu le sens sur tes doigts ? Oui, il colle. Le toit est bas, Raphaël. Oui, avec Chouchou. Le camion dort. L'odeur de résine reste sur la terrasse. Il est là, maman. Oui, sur le bord. L'éclat de planche tient sur le bord.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le camion a eu un garage. On a joué ensemble. Bravo, Raphaël. La planche sent encore la résine.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la caisse. Maman referme le bord, sans bruit. Comme un toit, papa. Tu le vois, toi ? Oui, sur le bord. On est bien, ici. Raphaël glisse le doigt, sans se presser. On le sent, maman. Tu le sens sur tes doigts ? Oui, il colle. Le toit est bas, Raphaël. Oui, avec Chouchou. Le camion dort. L'odeur de résine reste sur la terrasse. Il est là, maman. Oui, sur le bord. L'&lt;emphasis level="moderate"&gt;éclat de planche&lt;/emphasis&gt; tient sur le bord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la caisse. Maman referme le bord, sans bruit. Comme un toit, papa. Tu le vois, toi ? Oui, sur le bord. On est bien, ici. Raphaël glisse le doigt, sans se presser. On le sent, maman. Tu le sens sur tes doigts ? Oui, il colle. Le toit est bas, Raphaël. Oui, avec Chouchou. Le camion dort. L'odeur de résine reste sur la terrasse. Il est là, maman. Oui, sur le bord. L'&lt;emphasis&gt;éclat de planche&lt;/emphasis&gt; tient sur le bord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2011,15 +2104,15 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2031,12 +2124,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2045,17 +2138,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de planche</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2064,11 +2161,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2077,27 +2174,49 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bord; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|Le camion a eu un garage.
-enfant-m|On a joué ensemble.
-papa|Bravo, Raphaël.
-narrateur|La planche sent encore la résine.</t>
+          <t>narrateur|Ils restent près de la caisse.
+narrateur|Maman referme le bord, sans bruit.
+enfant-m|Comme un toit, papa.
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur le bord.
+maman|On est bien, ici.
+narrateur|Raphaël glisse le doigt, sans se presser.
+enfant-m|On le sent, maman.
+maman|Tu le sens sur tes doigts ?
+enfant-m|Oui, il colle.
+papa|Le toit est bas, Raphaël.
+enfant-m|Oui, avec Chouchou.
+enfant-f|Le camion dort.
+narrateur|L'odeur de résine reste sur la terrasse.
+enfant-m|Il est là, maman.
+maman|Oui, sur le bord.
+narrateur|L'éclat de planche tient sur le bord.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>linge</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2196,6 +2315,13 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>